<commit_message>
User stories for Immunisations Tab
</commit_message>
<xml_diff>
--- a/Business Analysis/checkupp_product_backlog.xlsx
+++ b/Business Analysis/checkupp_product_backlog.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Business Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CheckUpp\Business Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34550AD7-EA1C-44F2-8B37-D1E9B7DFAAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E11AF35-D9A5-4EBD-8DD3-E7EE2CBE1164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Tanvi_Immunisation_User_Stories" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$I$1:$I$32</definedName>
@@ -178,7 +179,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="374">
   <si>
     <t>Epic #</t>
   </si>
@@ -5299,12 +5300,1410 @@
 11. Zero Network Dependency (Privacy): Because scanning runs strictly via on-device ML Kit, the extraction feature must operate flawlessly when the device is fully offline, ensuring no visual data is transmitted over the internet.
 12. Lighting/Contrast Pre-Processing (Technical AC): Because floor scales are often highly reflective or backlit, the camera feed passed to ML Kit must utilize a threshold/contrast filter to isolate the glowing LCD numbers from the background glare.</t>
   </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>As a...</t>
+  </si>
+  <si>
+    <t>I want to...</t>
+  </si>
+  <si>
+    <t>So that...</t>
+  </si>
+  <si>
+    <t>Logged-in user navigating to the Immunisations screen</t>
+  </si>
+  <si>
+    <t>See the immunisation category relevant to my age bracket</t>
+  </si>
+  <si>
+    <t>I can easily identify vaccinations relevant to my current age group</t>
+  </si>
+  <si>
+    <t>Logged-in user whose profile indicates female gender and confirmed pregnancy</t>
+  </si>
+  <si>
+    <t>See pregnancy-specific immunisation recommendations</t>
+  </si>
+  <si>
+    <t>I can view vaccinations relevant to pregnancy</t>
+  </si>
+  <si>
+    <t>See vaccination recommendations personalised to my applicable age/life stage</t>
+  </si>
+  <si>
+    <t>I am not presented with irrelevant recommendations</t>
+  </si>
+  <si>
+    <t>Access the Travel immunisation category</t>
+  </si>
+  <si>
+    <t>I can view travel vaccination information regardless of my age or gender</t>
+  </si>
+  <si>
+    <t>Logged-in user who is at or above the defined legal parenting age</t>
+  </si>
+  <si>
+    <t>Access the Children immunisation category</t>
+  </si>
+  <si>
+    <t>I can view vaccination information relevant to children</t>
+  </si>
+  <si>
+    <t>Logged-in user browsing the Immunisations screen</t>
+  </si>
+  <si>
+    <t>Browse other applicable immunisation categories</t>
+  </si>
+  <si>
+    <t>I can access useful vaccination information beyond my personalised recommendations</t>
+  </si>
+  <si>
+    <t>Logged-in user selecting an immunisation category</t>
+  </si>
+  <si>
+    <t>View the vaccinations associated with that specific age group or life stage</t>
+  </si>
+  <si>
+    <t>I can understand which vaccinations belong to that category</t>
+  </si>
+  <si>
+    <t>Logged-in user viewing an immunisation category</t>
+  </si>
+  <si>
+    <t>View more information about an available vaccination</t>
+  </si>
+  <si>
+    <t>I can understand the vaccination recommendation presented to me</t>
+  </si>
+  <si>
+    <t>Logged-in user with incomplete or invalid profile information</t>
+  </si>
+  <si>
+    <t>See an appropriate Immunisations screen state</t>
+  </si>
+  <si>
+    <t>The interface does not provide incorrect personalised recommendations</t>
+  </si>
+  <si>
+    <t>Logged-in user using the Immunisations screen</t>
+  </si>
+  <si>
+    <t>See a consistent and usable immunisation interface</t>
+  </si>
+  <si>
+    <t>I can navigate recommendations and categories without confusion</t>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The frontend must determine the applicable age bracket using the user's configured age/test profile data.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The corresponding age-group card must be displayed in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recommended for You.
+3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Age-group labels and ranges must match the approved wireframe, e.g. Children, Adolescent, Adult, 50+ Years, 65+ Years and 70+ Years where applicable.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Age-group cards that are not applicable to the user must not appear in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recommended for You</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Boundary ages must map to the correct group according to the defined age ranges.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If age data is unavailable or invalid, age-specific recommendations must not be displayed and an appropriate frontend fallback message/state must be shown.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pregnancy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> card must be displayed when the configured user profile indicates both female gender </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>and</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> confirmed pregnancy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The Pregnancy card must not be displayed as a personalised recommendation when either condition is not satisfied.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Pregnancy recommendations must appear alongside any applicable age-based recommendation rather than replacing it.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Selecting the Pregnancy card must display the vaccination information configured for the pregnancy life stage.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The displayed Pregnancy card must follow the approved wireframe styling and interaction behaviour.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recommended for You</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must contain only cards applicable to the configured user profile.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The applicable age-based card must be displayed when valid age information is available.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A qualifying pregnant user must see both the applicable age-based recommendation and Pregnancy recommendation where both apply.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Non-applicable age/life-stage cards must not appear in this section.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Travel and other general browsing categories must not appear in Recommended for You unless separately defined as recommendations in the approved design.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The layout must correctly handle one or multiple recommendation cards without overlap, clipping, or broken spacing.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Travel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> card must always be displayed under </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Other Categories</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for every configured user profile.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Travel card visibility must not depend on age, gender, or pregnancy status.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Selecting the Travel card must display the configured travel vaccination information/list.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The Travel card must remain visible when testing different valid user profile combinations.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The card's label, description, icon and interaction must follow the approved wireframe.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Children (0–4 years)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> card must be displayed under </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Other Categories</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> when the configured user's age is </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>16 years or older</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The Children card must not be displayed when the configured user's age is below 16.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The boundary value of exactly 16 years must result in the Children card being displayed.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Visibility of the Children card must not depend on gender or pregnancy status.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Selecting the card must display the vaccination information configured for children aged 0–4 years.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Other Categories</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must be displayed separately from Recommended for You.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Cards within Other Categories must follow their defined frontend visibility rules.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Travel must be available to all users.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Children (0–4 years) must follow the 16+ visibility rule.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Pregnancy must follow its approved visibility rule for this section, if the product design includes Pregnancy under Other Categories.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Age/life-stage categories shown for general browsing must appear in the order specified by the approved wireframe.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>7.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Changes to the configured test profile must result in the appropriate category visibility changes when the screen is re-rendered.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Each category card must be associated with its approved vaccination list.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Selecting a card must display only the vaccination information configured for that category.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Vaccine names and accompanying frontend content must match the approved content source supplied to the development team.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Vaccines belonging exclusively to another category must not incorrectly appear in the selected category.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Categories containing multiple vaccines must display all configured vaccines without clipping or inaccessible content.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Empty or missing mock vaccination data must produce an appropriate frontend empty state rather than a blank or broken component.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Each displayed vaccination must be selectable where interaction is defined in the design.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Selecting a vaccination must display the corresponding configured details using the approved frontend component/screen.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The displayed vaccine information must correspond to the vaccination selected by the user.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The user must be able to return to the relevant immunisation category without breaking the screen state/navigation flow.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Missing optional information must not cause the component to crash or display malformed UI.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Missing/invalid age data must not result in an arbitrary age-specific recommendation being shown.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Missing pregnancy information must not cause the Pregnancy card to be treated as a personalised recommendation.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> General categories that do not depend on missing information, such as Travel, must remain accessible.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The frontend must display the defined fallback/empty state where personalised recommendations cannot be determined.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The screen must remain functional and must not crash because profile values are null, undefined, malformed, or otherwise unavailable.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recommended for You</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quick Actions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Other Categories</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> must appear in the order defined in the approved wireframe.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Cards must use consistent spacing, typography, icons, borders and interaction states according to the approved frontend design.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Conditional removal of a card must not leave unintended blank spaces or broken alignment.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Multiple Recommended for You cards must render correctly when more than one condition applies.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All visible interactive cards must respond to user selection and navigate/open the expected frontend content.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The screen must remain scrollable and all rendered content must be reachable on supported mobile screen sizes.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5426,6 +6825,13 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="19">
@@ -5624,7 +7030,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5797,6 +7203,72 @@
     <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5818,9 +7290,6 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5836,68 +7305,14 @@
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6116,50 +7531,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L94"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="64.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="72.5546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
-    <col min="10" max="12" width="8.88671875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.90625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="64.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="72.54296875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="11.6328125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.36328125" style="3" customWidth="1"/>
+    <col min="10" max="12" width="8.90625" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="74" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="74" t="s">
+      <c r="C1" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="74" t="s">
+      <c r="D1" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
       <c r="G1" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="74" t="s">
+      <c r="H1" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="74" t="s">
+      <c r="I1" s="71" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="65"/>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="64"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
       <c r="D2" s="4" t="s">
         <v>7</v>
       </c>
@@ -6170,10 +7585,10 @@
         <v>9</v>
       </c>
       <c r="G2" s="75"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-    </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+    </row>
+    <row r="3" spans="1:9" s="5" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="76">
         <v>1</v>
       </c>
@@ -6202,7 +7617,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="6" customFormat="1" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" s="6" customFormat="1" ht="124.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="76"/>
       <c r="B4" s="78"/>
       <c r="C4" s="16">
@@ -6223,7 +7638,7 @@
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
     </row>
-    <row r="5" spans="1:9" s="6" customFormat="1" ht="160.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" s="6" customFormat="1" ht="160.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="76"/>
       <c r="B5" s="78"/>
       <c r="C5" s="16">
@@ -6244,7 +7659,7 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:9" s="6" customFormat="1" ht="154.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" s="6" customFormat="1" ht="154.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="76"/>
       <c r="B6" s="78"/>
       <c r="C6" s="16">
@@ -6265,7 +7680,7 @@
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" spans="1:9" s="6" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" s="6" customFormat="1" ht="116" x14ac:dyDescent="0.35">
       <c r="A7" s="76"/>
       <c r="B7" s="78"/>
       <c r="C7" s="16">
@@ -6286,7 +7701,7 @@
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
     </row>
-    <row r="8" spans="1:9" s="6" customFormat="1" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" s="6" customFormat="1" ht="124.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="50"/>
       <c r="B8" s="78"/>
       <c r="C8" s="16">
@@ -6307,7 +7722,7 @@
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
     </row>
-    <row r="9" spans="1:9" s="6" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" s="6" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="50"/>
       <c r="B9" s="78"/>
       <c r="C9" s="16">
@@ -6328,7 +7743,7 @@
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
     </row>
-    <row r="10" spans="1:9" s="6" customFormat="1" ht="295.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" s="6" customFormat="1" ht="295.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="50"/>
       <c r="B10" s="79"/>
       <c r="C10" s="16">
@@ -6349,11 +7764,11 @@
       <c r="H10" s="16"/>
       <c r="I10" s="51"/>
     </row>
-    <row r="11" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="71">
+    <row r="11" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="72">
         <v>5</v>
       </c>
-      <c r="B11" s="71" t="s">
+      <c r="B11" s="72" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="18">
@@ -6378,9 +7793,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="72"/>
-      <c r="B12" s="72"/>
+    <row r="12" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="73"/>
+      <c r="B12" s="73"/>
       <c r="C12" s="18">
         <v>5.2</v>
       </c>
@@ -6399,9 +7814,9 @@
       <c r="H12" s="20"/>
       <c r="I12" s="18"/>
     </row>
-    <row r="13" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="72"/>
-      <c r="B13" s="72"/>
+    <row r="13" spans="1:9" s="6" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A13" s="73"/>
+      <c r="B13" s="73"/>
       <c r="C13" s="18">
         <v>5.3</v>
       </c>
@@ -6420,9 +7835,9 @@
       <c r="H13" s="20"/>
       <c r="I13" s="18"/>
     </row>
-    <row r="14" spans="1:9" s="14" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="72"/>
-      <c r="B14" s="72"/>
+    <row r="14" spans="1:9" s="14" customFormat="1" ht="232" x14ac:dyDescent="0.35">
+      <c r="A14" s="73"/>
+      <c r="B14" s="73"/>
       <c r="C14" s="21">
         <v>5.4</v>
       </c>
@@ -6441,9 +7856,9 @@
       <c r="H14" s="23"/>
       <c r="I14" s="21"/>
     </row>
-    <row r="15" spans="1:9" s="14" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="73"/>
-      <c r="B15" s="73"/>
+    <row r="15" spans="1:9" s="14" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A15" s="74"/>
+      <c r="B15" s="74"/>
       <c r="C15" s="21">
         <v>5.5</v>
       </c>
@@ -6462,11 +7877,11 @@
       <c r="H15" s="23"/>
       <c r="I15" s="21"/>
     </row>
-    <row r="16" spans="1:9" s="14" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="80">
+    <row r="16" spans="1:9" s="14" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A16" s="58">
         <v>6</v>
       </c>
-      <c r="B16" s="80" t="s">
+      <c r="B16" s="58" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="24">
@@ -6491,9 +7906,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A17" s="81"/>
-      <c r="B17" s="81"/>
+    <row r="17" spans="1:9" s="6" customFormat="1" ht="145" x14ac:dyDescent="0.35">
+      <c r="A17" s="59"/>
+      <c r="B17" s="59"/>
       <c r="C17" s="24">
         <v>6.2</v>
       </c>
@@ -6512,9 +7927,9 @@
       <c r="H17" s="26"/>
       <c r="I17" s="24"/>
     </row>
-    <row r="18" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="81"/>
-      <c r="B18" s="81"/>
+    <row r="18" spans="1:9" s="6" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A18" s="59"/>
+      <c r="B18" s="59"/>
       <c r="C18" s="24">
         <v>6.3</v>
       </c>
@@ -6533,9 +7948,9 @@
       <c r="H18" s="26"/>
       <c r="I18" s="24"/>
     </row>
-    <row r="19" spans="1:9" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="81"/>
-      <c r="B19" s="81"/>
+    <row r="19" spans="1:9" s="6" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="59"/>
+      <c r="B19" s="59"/>
       <c r="C19" s="27">
         <v>6.4</v>
       </c>
@@ -6558,9 +7973,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A20" s="52"/>
-      <c r="B20" s="81"/>
+      <c r="B20" s="59"/>
       <c r="C20" s="24">
         <v>6.5</v>
       </c>
@@ -6579,9 +7994,9 @@
       <c r="H20" s="26"/>
       <c r="I20" s="24"/>
     </row>
-    <row r="21" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A21" s="52"/>
-      <c r="B21" s="91"/>
+      <c r="B21" s="70"/>
       <c r="C21" s="24">
         <v>6.6</v>
       </c>
@@ -6600,11 +8015,11 @@
       <c r="H21" s="26"/>
       <c r="I21" s="24"/>
     </row>
-    <row r="22" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A22" s="82">
+    <row r="22" spans="1:9" s="6" customFormat="1" ht="145" x14ac:dyDescent="0.35">
+      <c r="A22" s="60">
         <v>7</v>
       </c>
-      <c r="B22" s="80" t="s">
+      <c r="B22" s="58" t="s">
         <v>34</v>
       </c>
       <c r="C22" s="24">
@@ -6629,9 +8044,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A23" s="83"/>
-      <c r="B23" s="81"/>
+    <row r="23" spans="1:9" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="61"/>
+      <c r="B23" s="59"/>
       <c r="C23" s="24">
         <v>7.2</v>
       </c>
@@ -6652,9 +8067,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="6" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="83"/>
-      <c r="B24" s="81"/>
+    <row r="24" spans="1:9" s="6" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="61"/>
+      <c r="B24" s="59"/>
       <c r="C24" s="24">
         <v>7.3</v>
       </c>
@@ -6673,9 +8088,9 @@
       <c r="H24" s="26"/>
       <c r="I24" s="24"/>
     </row>
-    <row r="25" spans="1:9" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="84"/>
-      <c r="B25" s="81"/>
+    <row r="25" spans="1:9" s="6" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="62"/>
+      <c r="B25" s="59"/>
       <c r="C25" s="24">
         <v>7.4</v>
       </c>
@@ -6694,9 +8109,9 @@
       <c r="H25" s="26"/>
       <c r="I25" s="24"/>
     </row>
-    <row r="26" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A26" s="52"/>
-      <c r="B26" s="91"/>
+      <c r="B26" s="70"/>
       <c r="C26" s="24">
         <v>7.5</v>
       </c>
@@ -6715,11 +8130,11 @@
       <c r="H26" s="26"/>
       <c r="I26" s="24"/>
     </row>
-    <row r="27" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="88">
+    <row r="27" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="67">
         <v>8</v>
       </c>
-      <c r="B27" s="88" t="s">
+      <c r="B27" s="67" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="28">
@@ -6742,9 +8157,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="89"/>
-      <c r="B28" s="89"/>
+    <row r="28" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="68"/>
+      <c r="B28" s="68"/>
       <c r="C28" s="28">
         <v>9.3000000000000007</v>
       </c>
@@ -6765,9 +8180,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="90"/>
-      <c r="B29" s="90"/>
+    <row r="29" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="69"/>
+      <c r="B29" s="69"/>
       <c r="C29" s="28">
         <v>9.4</v>
       </c>
@@ -6788,11 +8203,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="86">
+    <row r="30" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A30" s="65">
         <v>12</v>
       </c>
-      <c r="B30" s="86" t="s">
+      <c r="B30" s="65" t="s">
         <v>54</v>
       </c>
       <c r="C30" s="30">
@@ -6817,9 +8232,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="86"/>
-      <c r="B31" s="86"/>
+    <row r="31" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A31" s="65"/>
+      <c r="B31" s="65"/>
       <c r="C31" s="30">
         <v>12.2</v>
       </c>
@@ -6842,9 +8257,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="86"/>
-      <c r="B32" s="86"/>
+    <row r="32" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="65"/>
+      <c r="B32" s="65"/>
       <c r="C32" s="30">
         <v>12.3</v>
       </c>
@@ -6867,9 +8282,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:9" s="6" customFormat="1" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="86"/>
-      <c r="B33" s="86"/>
+    <row r="33" spans="1:9" s="6" customFormat="1" ht="123.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="65"/>
+      <c r="B33" s="65"/>
       <c r="C33" s="30">
         <v>12.4</v>
       </c>
@@ -6892,9 +8307,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="86"/>
-      <c r="B34" s="86"/>
+    <row r="34" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="65"/>
+      <c r="B34" s="65"/>
       <c r="C34" s="30">
         <v>12.5</v>
       </c>
@@ -6917,11 +8332,11 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="87">
+    <row r="35" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="66">
         <v>14</v>
       </c>
-      <c r="B35" s="87" t="s">
+      <c r="B35" s="66" t="s">
         <v>70</v>
       </c>
       <c r="C35" s="34">
@@ -6946,9 +8361,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="87"/>
-      <c r="B36" s="87"/>
+    <row r="36" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="66"/>
+      <c r="B36" s="66"/>
       <c r="C36" s="34">
         <v>14.2</v>
       </c>
@@ -6971,9 +8386,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="87"/>
-      <c r="B37" s="87"/>
+    <row r="37" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="66"/>
+      <c r="B37" s="66"/>
       <c r="C37" s="34">
         <v>14.3</v>
       </c>
@@ -6996,9 +8411,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="87"/>
-      <c r="B38" s="87"/>
+    <row r="38" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A38" s="66"/>
+      <c r="B38" s="66"/>
       <c r="C38" s="34">
         <v>14.4</v>
       </c>
@@ -7021,9 +8436,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="87"/>
-      <c r="B39" s="87"/>
+    <row r="39" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="66"/>
+      <c r="B39" s="66"/>
       <c r="C39" s="34">
         <v>14.5</v>
       </c>
@@ -7046,9 +8461,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="87"/>
-      <c r="B40" s="87"/>
+    <row r="40" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="66"/>
+      <c r="B40" s="66"/>
       <c r="C40" s="34">
         <v>14.6</v>
       </c>
@@ -7071,9 +8486,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="87"/>
-      <c r="B41" s="87"/>
+    <row r="41" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="66"/>
+      <c r="B41" s="66"/>
       <c r="C41" s="34">
         <v>14.7</v>
       </c>
@@ -7096,9 +8511,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="87"/>
-      <c r="B42" s="87"/>
+    <row r="42" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="66"/>
+      <c r="B42" s="66"/>
       <c r="C42" s="34">
         <v>14.8</v>
       </c>
@@ -7121,9 +8536,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="87"/>
-      <c r="B43" s="87"/>
+    <row r="43" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A43" s="66"/>
+      <c r="B43" s="66"/>
       <c r="C43" s="34">
         <v>14.9</v>
       </c>
@@ -7146,9 +8561,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="44" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="87"/>
-      <c r="B44" s="87"/>
+    <row r="44" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A44" s="66"/>
+      <c r="B44" s="66"/>
       <c r="C44" s="34">
         <v>14.1</v>
       </c>
@@ -7171,9 +8586,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="45" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="87"/>
-      <c r="B45" s="87"/>
+    <row r="45" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="66"/>
+      <c r="B45" s="66"/>
       <c r="C45" s="34">
         <v>14.11</v>
       </c>
@@ -7196,11 +8611,11 @@
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="85">
+    <row r="46" spans="1:9" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A46" s="63">
         <v>15</v>
       </c>
-      <c r="B46" s="85" t="s">
+      <c r="B46" s="63" t="s">
         <v>74</v>
       </c>
       <c r="C46" s="37">
@@ -7225,9 +8640,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="47" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="65"/>
-      <c r="B47" s="65"/>
+    <row r="47" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A47" s="64"/>
+      <c r="B47" s="64"/>
       <c r="C47" s="37">
         <v>15.2</v>
       </c>
@@ -7250,9 +8665,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="65"/>
-      <c r="B48" s="65"/>
+    <row r="48" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A48" s="64"/>
+      <c r="B48" s="64"/>
       <c r="C48" s="37">
         <v>15.3</v>
       </c>
@@ -7275,9 +8690,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="49" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="65"/>
-      <c r="B49" s="65"/>
+    <row r="49" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A49" s="64"/>
+      <c r="B49" s="64"/>
       <c r="C49" s="37">
         <v>15.4</v>
       </c>
@@ -7300,9 +8715,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="65"/>
-      <c r="B50" s="65"/>
+    <row r="50" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A50" s="64"/>
+      <c r="B50" s="64"/>
       <c r="C50" s="37">
         <v>15.5</v>
       </c>
@@ -7325,9 +8740,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="65"/>
-      <c r="B51" s="65"/>
+    <row r="51" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A51" s="64"/>
+      <c r="B51" s="64"/>
       <c r="C51" s="37">
         <v>15.6</v>
       </c>
@@ -7350,9 +8765,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A52" s="65"/>
-      <c r="B52" s="65"/>
+    <row r="52" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A52" s="64"/>
+      <c r="B52" s="64"/>
       <c r="C52" s="37">
         <v>15.7</v>
       </c>
@@ -7375,9 +8790,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="53" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="65"/>
-      <c r="B53" s="65"/>
+    <row r="53" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A53" s="64"/>
+      <c r="B53" s="64"/>
       <c r="C53" s="37">
         <v>15.8</v>
       </c>
@@ -7400,11 +8815,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="54" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="64">
+    <row r="54" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A54" s="86">
         <v>16</v>
       </c>
-      <c r="B54" s="64" t="s">
+      <c r="B54" s="86" t="s">
         <v>89</v>
       </c>
       <c r="C54" s="39">
@@ -7429,9 +8844,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="55" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="64"/>
-      <c r="B55" s="64"/>
+    <row r="55" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A55" s="86"/>
+      <c r="B55" s="86"/>
       <c r="C55" s="39">
         <v>16.2</v>
       </c>
@@ -7454,9 +8869,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="56" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="64"/>
-      <c r="B56" s="64"/>
+    <row r="56" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A56" s="86"/>
+      <c r="B56" s="86"/>
       <c r="C56" s="39">
         <v>16.3</v>
       </c>
@@ -7479,9 +8894,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="57" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="64"/>
-      <c r="B57" s="64"/>
+    <row r="57" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A57" s="86"/>
+      <c r="B57" s="86"/>
       <c r="C57" s="39">
         <v>16.399999999999999</v>
       </c>
@@ -7504,9 +8919,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="58" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="64"/>
-      <c r="B58" s="64"/>
+    <row r="58" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A58" s="86"/>
+      <c r="B58" s="86"/>
       <c r="C58" s="39">
         <v>16.5</v>
       </c>
@@ -7529,9 +8944,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="59" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="65"/>
-      <c r="B59" s="65"/>
+    <row r="59" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A59" s="64"/>
+      <c r="B59" s="64"/>
       <c r="C59" s="39">
         <v>16.600000000000001</v>
       </c>
@@ -7554,11 +8969,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="60" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="66">
+    <row r="60" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A60" s="87">
         <v>17</v>
       </c>
-      <c r="B60" s="69" t="s">
+      <c r="B60" s="90" t="s">
         <v>105</v>
       </c>
       <c r="C60" s="42">
@@ -7583,9 +8998,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="61" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="67"/>
-      <c r="B61" s="69"/>
+    <row r="61" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A61" s="88"/>
+      <c r="B61" s="90"/>
       <c r="C61" s="42">
         <v>17.2</v>
       </c>
@@ -7608,9 +9023,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="62" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="67"/>
-      <c r="B62" s="69"/>
+    <row r="62" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="88"/>
+      <c r="B62" s="90"/>
       <c r="C62" s="42">
         <v>17.3</v>
       </c>
@@ -7633,9 +9048,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A63" s="67"/>
-      <c r="B63" s="69"/>
+    <row r="63" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A63" s="88"/>
+      <c r="B63" s="90"/>
       <c r="C63" s="42">
         <v>17.399999999999999</v>
       </c>
@@ -7658,9 +9073,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="64" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A64" s="68"/>
-      <c r="B64" s="69"/>
+    <row r="64" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A64" s="89"/>
+      <c r="B64" s="90"/>
       <c r="C64" s="42">
         <v>17.5</v>
       </c>
@@ -7683,11 +9098,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="65" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="70">
+    <row r="65" spans="1:12" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A65" s="91">
         <v>18</v>
       </c>
-      <c r="B65" s="71" t="s">
+      <c r="B65" s="72" t="s">
         <v>279</v>
       </c>
       <c r="C65" s="18">
@@ -7712,9 +9127,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="66" spans="1:12" s="6" customFormat="1" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="65"/>
-      <c r="B66" s="72"/>
+    <row r="66" spans="1:12" s="6" customFormat="1" ht="250.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="64"/>
+      <c r="B66" s="73"/>
       <c r="C66" s="18">
         <v>18.2</v>
       </c>
@@ -7737,9 +9152,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="6" customFormat="1" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="65"/>
-      <c r="B67" s="72"/>
+    <row r="67" spans="1:12" s="6" customFormat="1" ht="167.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="64"/>
+      <c r="B67" s="73"/>
       <c r="C67" s="18">
         <v>18.3</v>
       </c>
@@ -7762,9 +9177,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="68" spans="1:12" s="6" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A68" s="65"/>
-      <c r="B68" s="72"/>
+    <row r="68" spans="1:12" s="6" customFormat="1" ht="246.5" x14ac:dyDescent="0.35">
+      <c r="A68" s="64"/>
+      <c r="B68" s="73"/>
       <c r="C68" s="18">
         <v>18.399999999999999</v>
       </c>
@@ -7787,9 +9202,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="6" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" s="6" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="48"/>
-      <c r="B69" s="73"/>
+      <c r="B69" s="74"/>
       <c r="C69" s="18">
         <v>18.5</v>
       </c>
@@ -7808,11 +9223,11 @@
       <c r="H69" s="18"/>
       <c r="I69" s="18"/>
     </row>
-    <row r="70" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="58">
+    <row r="70" spans="1:12" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A70" s="80">
         <v>19</v>
       </c>
-      <c r="B70" s="61" t="s">
+      <c r="B70" s="83" t="s">
         <v>120</v>
       </c>
       <c r="C70" s="44">
@@ -7833,9 +9248,9 @@
       <c r="H70" s="44"/>
       <c r="I70" s="47"/>
     </row>
-    <row r="71" spans="1:12" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="59"/>
-      <c r="B71" s="62"/>
+    <row r="71" spans="1:12" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A71" s="81"/>
+      <c r="B71" s="84"/>
       <c r="C71" s="15">
         <v>19.2</v>
       </c>
@@ -7854,9 +9269,9 @@
       <c r="H71" s="44"/>
       <c r="I71" s="47"/>
     </row>
-    <row r="72" spans="1:12" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="60"/>
-      <c r="B72" s="63"/>
+    <row r="72" spans="1:12" s="6" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A72" s="82"/>
+      <c r="B72" s="85"/>
       <c r="C72" s="53">
         <v>19.3</v>
       </c>
@@ -7877,11 +9292,11 @@
         <v>313</v>
       </c>
     </row>
-    <row r="73" spans="1:12" s="6" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A73" s="58">
+    <row r="73" spans="1:12" s="6" customFormat="1" ht="203" x14ac:dyDescent="0.35">
+      <c r="A73" s="80">
         <v>20</v>
       </c>
-      <c r="B73" s="61" t="s">
+      <c r="B73" s="83" t="s">
         <v>126</v>
       </c>
       <c r="C73" s="44">
@@ -7902,9 +9317,9 @@
       <c r="H73" s="44"/>
       <c r="I73" s="47"/>
     </row>
-    <row r="74" spans="1:12" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="59"/>
-      <c r="B74" s="62"/>
+    <row r="74" spans="1:12" s="6" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A74" s="81"/>
+      <c r="B74" s="84"/>
       <c r="C74" s="15">
         <v>20.2</v>
       </c>
@@ -7926,9 +9341,9 @@
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
     </row>
-    <row r="75" spans="1:12" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A75" s="60"/>
-      <c r="B75" s="62"/>
+    <row r="75" spans="1:12" s="6" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A75" s="82"/>
+      <c r="B75" s="84"/>
       <c r="C75" s="56">
         <v>20.3</v>
       </c>
@@ -7952,9 +9367,9 @@
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
     </row>
-    <row r="76" spans="1:12" s="6" customFormat="1" ht="331.2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" s="6" customFormat="1" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A76" s="49"/>
-      <c r="B76" s="63"/>
+      <c r="B76" s="85"/>
       <c r="C76" s="56">
         <v>20.399999999999999</v>
       </c>
@@ -7978,11 +9393,11 @@
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
     </row>
-    <row r="77" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="58">
+    <row r="77" spans="1:12" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A77" s="80">
         <v>21</v>
       </c>
-      <c r="B77" s="61" t="s">
+      <c r="B77" s="83" t="s">
         <v>129</v>
       </c>
       <c r="C77" s="44">
@@ -8003,9 +9418,9 @@
       <c r="H77" s="44"/>
       <c r="I77" s="47"/>
     </row>
-    <row r="78" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="59"/>
-      <c r="B78" s="62"/>
+    <row r="78" spans="1:12" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A78" s="81"/>
+      <c r="B78" s="84"/>
       <c r="C78" s="15">
         <v>21.2</v>
       </c>
@@ -8024,9 +9439,9 @@
       <c r="H78" s="44"/>
       <c r="I78" s="47"/>
     </row>
-    <row r="79" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A79" s="60"/>
-      <c r="B79" s="63"/>
+    <row r="79" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A79" s="82"/>
+      <c r="B79" s="85"/>
       <c r="C79" s="32">
         <v>21.3</v>
       </c>
@@ -8041,11 +9456,11 @@
       <c r="H79" s="32"/>
       <c r="I79" s="33"/>
     </row>
-    <row r="80" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A80" s="58">
+    <row r="80" spans="1:12" ht="261" x14ac:dyDescent="0.35">
+      <c r="A80" s="80">
         <v>22</v>
       </c>
-      <c r="B80" s="61" t="s">
+      <c r="B80" s="83" t="s">
         <v>133</v>
       </c>
       <c r="C80" s="44">
@@ -8066,9 +9481,9 @@
       <c r="H80" s="44"/>
       <c r="I80" s="47"/>
     </row>
-    <row r="81" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A81" s="59"/>
-      <c r="B81" s="62"/>
+    <row r="81" spans="1:9" ht="261" x14ac:dyDescent="0.35">
+      <c r="A81" s="81"/>
+      <c r="B81" s="84"/>
       <c r="C81" s="15">
         <v>22.2</v>
       </c>
@@ -8087,9 +9502,9 @@
       <c r="H81" s="44"/>
       <c r="I81" s="47"/>
     </row>
-    <row r="82" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A82" s="60"/>
-      <c r="B82" s="63"/>
+    <row r="82" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A82" s="82"/>
+      <c r="B82" s="85"/>
       <c r="C82" s="32">
         <v>22.3</v>
       </c>
@@ -8104,26 +9519,26 @@
       <c r="H82" s="32"/>
       <c r="I82" s="33"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="E83" s="11"/>
       <c r="H83" s="3"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="I84" s="2"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
       <c r="I85" s="2"/>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" s="7"/>
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
@@ -8134,7 +9549,7 @@
       <c r="H86" s="7"/>
       <c r="I86" s="7"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -8145,7 +9560,7 @@
       <c r="H87" s="10"/>
       <c r="I87" s="10"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D88" s="10"/>
       <c r="E88" s="10"/>
       <c r="F88" s="10"/>
@@ -8153,7 +9568,7 @@
       <c r="H88" s="10"/>
       <c r="I88" s="10"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="D89" s="10"/>
       <c r="E89" s="10"/>
@@ -8162,7 +9577,7 @@
       <c r="H89" s="10"/>
       <c r="I89" s="10"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D90" s="10"/>
       <c r="E90" s="10"/>
       <c r="F90" s="10"/>
@@ -8170,7 +9585,7 @@
       <c r="H90" s="10"/>
       <c r="I90" s="10"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D91" s="10"/>
       <c r="E91" s="10"/>
       <c r="F91" s="10"/>
@@ -8178,7 +9593,7 @@
       <c r="H91" s="10"/>
       <c r="I91" s="10"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D92" s="10"/>
       <c r="E92" s="10"/>
       <c r="F92" s="10"/>
@@ -8186,7 +9601,7 @@
       <c r="H92" s="10"/>
       <c r="I92" s="10"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D93" s="10"/>
       <c r="E93" s="10"/>
       <c r="F93" s="10"/>
@@ -8194,7 +9609,7 @@
       <c r="H93" s="10"/>
       <c r="I93" s="10"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D94" s="10"/>
       <c r="E94" s="10"/>
       <c r="F94" s="10"/>
@@ -8205,29 +9620,6 @@
   </sheetData>
   <autoFilter ref="I1:I32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="37">
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A46:A53"/>
-    <mergeCell ref="B46:B53"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="A35:A45"/>
-    <mergeCell ref="B35:B45"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B26"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B10"/>
     <mergeCell ref="A77:A79"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A80:A82"/>
@@ -8242,6 +9634,29 @@
     <mergeCell ref="A73:A75"/>
     <mergeCell ref="B73:B76"/>
     <mergeCell ref="B65:B69"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B10"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A46:A53"/>
+    <mergeCell ref="B46:B53"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A35:A45"/>
+    <mergeCell ref="B35:B45"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B26"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8253,15 +9668,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="18.21875" customWidth="1"/>
-    <col min="5" max="5" width="24.88671875" customWidth="1"/>
-    <col min="6" max="6" width="27.33203125" customWidth="1"/>
-    <col min="7" max="7" width="36.21875" customWidth="1"/>
+    <col min="4" max="4" width="18.1796875" customWidth="1"/>
+    <col min="5" max="5" width="24.90625" customWidth="1"/>
+    <col min="6" max="6" width="27.36328125" customWidth="1"/>
+    <col min="7" max="7" width="36.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="9"/>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -8273,7 +9688,7 @@
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="9"/>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
@@ -8285,7 +9700,7 @@
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
     </row>
-    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -8309,7 +9724,7 @@
       </c>
       <c r="J3" s="9"/>
     </row>
-    <row r="4" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="348" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -8333,7 +9748,7 @@
       </c>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -8357,7 +9772,7 @@
       </c>
       <c r="J5" s="9"/>
     </row>
-    <row r="6" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="348" x14ac:dyDescent="0.35">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -8381,7 +9796,7 @@
       </c>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:10" ht="403.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="406" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -8405,7 +9820,7 @@
       </c>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -8429,7 +9844,7 @@
       </c>
       <c r="J8" s="9"/>
     </row>
-    <row r="9" spans="1:10" ht="273.60000000000002" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -8453,7 +9868,7 @@
       </c>
       <c r="J9" s="9"/>
     </row>
-    <row r="10" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="348" x14ac:dyDescent="0.35">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -8477,7 +9892,7 @@
       </c>
       <c r="J10" s="9"/>
     </row>
-    <row r="11" spans="1:10" ht="316.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="319" x14ac:dyDescent="0.35">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -8501,7 +9916,7 @@
       </c>
       <c r="J11" s="9"/>
     </row>
-    <row r="12" spans="1:10" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -8525,7 +9940,7 @@
       </c>
       <c r="J12" s="9"/>
     </row>
-    <row r="13" spans="1:10" ht="388.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -8549,7 +9964,7 @@
       </c>
       <c r="J13" s="9"/>
     </row>
-    <row r="14" spans="1:10" ht="288" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="290" x14ac:dyDescent="0.35">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -8573,7 +9988,7 @@
       </c>
       <c r="J14" s="9"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -8585,7 +10000,7 @@
       <c r="I15" s="9"/>
       <c r="J15" s="9"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -8597,7 +10012,7 @@
       <c r="I16" s="9"/>
       <c r="J16" s="9"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -8609,7 +10024,7 @@
       <c r="I17" s="9"/>
       <c r="J17" s="9"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -8621,7 +10036,7 @@
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -8633,7 +10048,7 @@
       <c r="I19" s="9"/>
       <c r="J19" s="9"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -8645,7 +10060,7 @@
       <c r="I20" s="9"/>
       <c r="J20" s="9"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -8657,7 +10072,7 @@
       <c r="I21" s="9"/>
       <c r="J21" s="9"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -8669,7 +10084,7 @@
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -8681,7 +10096,7 @@
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -8693,7 +10108,7 @@
       <c r="I24" s="9"/>
       <c r="J24" s="9"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -8705,7 +10120,7 @@
       <c r="I25" s="9"/>
       <c r="J25" s="9"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -8717,7 +10132,7 @@
       <c r="I26" s="9"/>
       <c r="J26" s="9"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -8729,7 +10144,7 @@
       <c r="I27" s="9"/>
       <c r="J27" s="9"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -8741,7 +10156,7 @@
       <c r="I28" s="9"/>
       <c r="J28" s="9"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -8753,7 +10168,7 @@
       <c r="I29" s="9"/>
       <c r="J29" s="9"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -8765,7 +10180,7 @@
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -8777,7 +10192,7 @@
       <c r="I31" s="9"/>
       <c r="J31" s="9"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -8789,63 +10204,63 @@
       <c r="I32" s="9"/>
       <c r="J32" s="9"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="9"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
@@ -8856,4 +10271,208 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0802363A-09BC-4F89-B136-783D2DDEAFD1}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21.7265625" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" customWidth="1"/>
+    <col min="3" max="3" width="55.1796875" customWidth="1"/>
+    <col min="4" max="4" width="70.26953125" customWidth="1"/>
+    <col min="5" max="5" width="89.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="92" t="s">
+        <v>332</v>
+      </c>
+      <c r="B1" s="92" t="s">
+        <v>333</v>
+      </c>
+      <c r="C1" s="92" t="s">
+        <v>334</v>
+      </c>
+      <c r="D1" s="92" t="s">
+        <v>335</v>
+      </c>
+      <c r="E1" s="92" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="203" x14ac:dyDescent="0.35">
+      <c r="A2" s="93">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="E2" s="93" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A3" s="93">
+        <v>5.2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>341</v>
+      </c>
+      <c r="E3" s="93" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="174" x14ac:dyDescent="0.35">
+      <c r="A4" s="93">
+        <v>5.3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>343</v>
+      </c>
+      <c r="E4" s="93" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="93">
+        <v>5.4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>336</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="E5" s="93" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="93">
+        <v>5.5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>348</v>
+      </c>
+      <c r="E6" s="93" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="174" x14ac:dyDescent="0.35">
+      <c r="A7" s="93">
+        <v>5.6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>349</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="E7" s="93" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="93">
+        <v>5.7</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>353</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="E8" s="93" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A9" s="93">
+        <v>5.8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>356</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>357</v>
+      </c>
+      <c r="E9" s="93" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A10" s="93">
+        <v>5.9</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="E10" s="93" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A11" s="94">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="E11" s="93" t="s">
+        <v>373</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated User stories for Immunisations Tab
</commit_message>
<xml_diff>
--- a/Business Analysis/checkupp_product_backlog.xlsx
+++ b/Business Analysis/checkupp_product_backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\CheckUpp\Business Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CheckUpp\Business Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25CAF1AC-1AFC-4D00-884A-F47A2BAA0FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443E0692-E891-49C3-BE56-000C29AAC3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6577,14 +6577,18 @@
     </r>
   </si>
   <si>
+    <t>I can access which vaccinations belong to that category</t>
+  </si>
+  <si>
     <r>
       <t>1.</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The </t>
@@ -6593,8 +6597,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Children (0–4 years)</t>
@@ -6602,8 +6607,9 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> card must be displayed under </t>
@@ -6612,8 +6618,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Other Categories</t>
@@ -6621,8 +6628,9 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> when the configured user's age is </t>
@@ -6631,8 +6639,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>16 years or older</t>
@@ -6640,8 +6649,9 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">.
@@ -6651,8 +6661,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>2.</t>
@@ -6660,8 +6671,9 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The Children card must not be displayed when the configured user's age is below 16.
@@ -6671,8 +6683,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>3.</t>
@@ -6680,8 +6693,9 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The boundary value of exactly 16 years must result in the Children card being displayed.
@@ -6691,8 +6705,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>4.</t>
@@ -6700,8 +6715,9 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> Visibility of the Children card must not depend on gender or pregnancy status.
@@ -6711,8 +6727,9 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>5.</t>
@@ -6720,11 +6737,45 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> Selecting the card must display the vaccination information configured for children aged 0–4 years.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Must be obscured in MVP.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
   </si>
   <si>
@@ -6819,7 +6870,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Children (0–4 years) must follow the 16+ visibility rule.</t>
+      <t xml:space="preserve"> Children (0–4 years) must follow the 16+ visibility rule</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. (Must be obscured in MVP)</t>
     </r>
     <r>
       <rPr>
@@ -6874,16 +6936,13 @@
       </rPr>
       <t xml:space="preserve"> Changes to the configured test profile must result in the appropriate category visibility changes when the screen is re-rendered.</t>
     </r>
-  </si>
-  <si>
-    <t>I can access which vaccinations belong to that category</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7062,6 +7121,28 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="21">
@@ -7460,9 +7541,6 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -7476,72 +7554,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -7565,6 +7577,9 @@
     <xf numFmtId="0" fontId="16" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7579,6 +7594,72 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7797,47 +7878,47 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L94"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="64.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="72.5546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
-    <col min="10" max="12" width="8.88671875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="5.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.90625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="64.90625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="72.54296875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="11.6328125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.36328125" style="3" customWidth="1"/>
+    <col min="10" max="12" width="8.90625" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="82" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="82" t="s">
+      <c r="B1" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="82" t="s">
+      <c r="C1" s="84" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="82" t="s">
+      <c r="D1" s="84" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="75"/>
       <c r="F1" s="75"/>
-      <c r="G1" s="86" t="s">
+      <c r="G1" s="85" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="82" t="s">
+      <c r="H1" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="82" t="s">
+      <c r="I1" s="84" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="75"/>
       <c r="B2" s="75"/>
       <c r="C2" s="75"/>
@@ -7850,15 +7931,15 @@
       <c r="F2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="86"/>
+      <c r="G2" s="85"/>
       <c r="H2" s="75"/>
       <c r="I2" s="75"/>
     </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="87">
+    <row r="3" spans="1:9" s="5" customFormat="1" ht="108" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="86">
         <v>1</v>
       </c>
-      <c r="B3" s="88" t="s">
+      <c r="B3" s="87" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="16">
@@ -7883,9 +7964,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="6" customFormat="1" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="87"/>
-      <c r="B4" s="89"/>
+    <row r="4" spans="1:9" s="6" customFormat="1" ht="124.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="86"/>
+      <c r="B4" s="88"/>
       <c r="C4" s="16">
         <v>1.2</v>
       </c>
@@ -7904,9 +7985,9 @@
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
     </row>
-    <row r="5" spans="1:9" s="6" customFormat="1" ht="160.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="87"/>
-      <c r="B5" s="89"/>
+    <row r="5" spans="1:9" s="6" customFormat="1" ht="160.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="86"/>
+      <c r="B5" s="88"/>
       <c r="C5" s="16">
         <v>1.3</v>
       </c>
@@ -7925,9 +8006,9 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:9" s="6" customFormat="1" ht="154.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="87"/>
-      <c r="B6" s="89"/>
+    <row r="6" spans="1:9" s="6" customFormat="1" ht="154.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="86"/>
+      <c r="B6" s="88"/>
       <c r="C6" s="16">
         <v>1.4</v>
       </c>
@@ -7946,9 +8027,9 @@
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" spans="1:9" s="6" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="87"/>
-      <c r="B7" s="89"/>
+    <row r="7" spans="1:9" s="6" customFormat="1" ht="116" x14ac:dyDescent="0.35">
+      <c r="A7" s="86"/>
+      <c r="B7" s="88"/>
       <c r="C7" s="16">
         <v>1.5</v>
       </c>
@@ -7967,9 +8048,9 @@
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
     </row>
-    <row r="8" spans="1:9" s="6" customFormat="1" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" s="6" customFormat="1" ht="124.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="50"/>
-      <c r="B8" s="89"/>
+      <c r="B8" s="88"/>
       <c r="C8" s="16">
         <v>1.6</v>
       </c>
@@ -7988,9 +8069,9 @@
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
     </row>
-    <row r="9" spans="1:9" s="6" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" s="6" customFormat="1" ht="152.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="50"/>
-      <c r="B9" s="89"/>
+      <c r="B9" s="88"/>
       <c r="C9" s="16">
         <v>1.7</v>
       </c>
@@ -8009,9 +8090,9 @@
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
     </row>
-    <row r="10" spans="1:9" s="6" customFormat="1" ht="295.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" s="6" customFormat="1" ht="295.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="50"/>
-      <c r="B10" s="90"/>
+      <c r="B10" s="89"/>
       <c r="C10" s="16">
         <v>1.8</v>
       </c>
@@ -8030,11 +8111,11 @@
       <c r="H10" s="16"/>
       <c r="I10" s="51"/>
     </row>
-    <row r="11" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="83">
+    <row r="11" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="81">
         <v>5</v>
       </c>
-      <c r="B11" s="83" t="s">
+      <c r="B11" s="81" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="18">
@@ -8059,9 +8140,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="84"/>
-      <c r="B12" s="84"/>
+    <row r="12" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A12" s="82"/>
+      <c r="B12" s="82"/>
       <c r="C12" s="18">
         <v>5.2</v>
       </c>
@@ -8080,9 +8161,9 @@
       <c r="H12" s="20"/>
       <c r="I12" s="18"/>
     </row>
-    <row r="13" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="84"/>
-      <c r="B13" s="84"/>
+    <row r="13" spans="1:9" s="6" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A13" s="82"/>
+      <c r="B13" s="82"/>
       <c r="C13" s="18">
         <v>5.3</v>
       </c>
@@ -8101,9 +8182,9 @@
       <c r="H13" s="20"/>
       <c r="I13" s="18"/>
     </row>
-    <row r="14" spans="1:9" s="14" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="84"/>
-      <c r="B14" s="84"/>
+    <row r="14" spans="1:9" s="14" customFormat="1" ht="232" x14ac:dyDescent="0.35">
+      <c r="A14" s="82"/>
+      <c r="B14" s="82"/>
       <c r="C14" s="21">
         <v>5.4</v>
       </c>
@@ -8122,9 +8203,9 @@
       <c r="H14" s="23"/>
       <c r="I14" s="21"/>
     </row>
-    <row r="15" spans="1:9" s="14" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="85"/>
-      <c r="B15" s="85"/>
+    <row r="15" spans="1:9" s="14" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A15" s="83"/>
+      <c r="B15" s="83"/>
       <c r="C15" s="21">
         <v>5.5</v>
       </c>
@@ -8143,11 +8224,11 @@
       <c r="H15" s="23"/>
       <c r="I15" s="21"/>
     </row>
-    <row r="16" spans="1:9" s="14" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="69">
+    <row r="16" spans="1:9" s="14" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A16" s="90">
         <v>6</v>
       </c>
-      <c r="B16" s="69" t="s">
+      <c r="B16" s="90" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="24">
@@ -8172,9 +8253,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A17" s="70"/>
-      <c r="B17" s="70"/>
+    <row r="17" spans="1:9" s="6" customFormat="1" ht="145" x14ac:dyDescent="0.35">
+      <c r="A17" s="91"/>
+      <c r="B17" s="91"/>
       <c r="C17" s="24">
         <v>6.2</v>
       </c>
@@ -8193,9 +8274,9 @@
       <c r="H17" s="26"/>
       <c r="I17" s="24"/>
     </row>
-    <row r="18" spans="1:9" s="6" customFormat="1" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="70"/>
-      <c r="B18" s="70"/>
+    <row r="18" spans="1:9" s="6" customFormat="1" ht="174" x14ac:dyDescent="0.35">
+      <c r="A18" s="91"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="24">
         <v>6.3</v>
       </c>
@@ -8214,9 +8295,9 @@
       <c r="H18" s="26"/>
       <c r="I18" s="24"/>
     </row>
-    <row r="19" spans="1:9" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="70"/>
-      <c r="B19" s="70"/>
+    <row r="19" spans="1:9" s="6" customFormat="1" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="91"/>
+      <c r="B19" s="91"/>
       <c r="C19" s="27">
         <v>6.4</v>
       </c>
@@ -8239,9 +8320,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
       <c r="A20" s="52"/>
-      <c r="B20" s="70"/>
+      <c r="B20" s="91"/>
       <c r="C20" s="24">
         <v>6.5</v>
       </c>
@@ -8260,9 +8341,9 @@
       <c r="H20" s="26"/>
       <c r="I20" s="24"/>
     </row>
-    <row r="21" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A21" s="52"/>
-      <c r="B21" s="81"/>
+      <c r="B21" s="101"/>
       <c r="C21" s="24">
         <v>6.6</v>
       </c>
@@ -8281,11 +8362,11 @@
       <c r="H21" s="26"/>
       <c r="I21" s="24"/>
     </row>
-    <row r="22" spans="1:9" s="6" customFormat="1" ht="144" x14ac:dyDescent="0.3">
-      <c r="A22" s="71">
+    <row r="22" spans="1:9" s="6" customFormat="1" ht="145" x14ac:dyDescent="0.35">
+      <c r="A22" s="92">
         <v>7</v>
       </c>
-      <c r="B22" s="69" t="s">
+      <c r="B22" s="90" t="s">
         <v>34</v>
       </c>
       <c r="C22" s="24">
@@ -8310,9 +8391,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
-      <c r="A23" s="72"/>
-      <c r="B23" s="70"/>
+    <row r="23" spans="1:9" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="93"/>
+      <c r="B23" s="91"/>
       <c r="C23" s="24">
         <v>7.2</v>
       </c>
@@ -8333,9 +8414,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="6" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="72"/>
-      <c r="B24" s="70"/>
+    <row r="24" spans="1:9" s="6" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="93"/>
+      <c r="B24" s="91"/>
       <c r="C24" s="24">
         <v>7.3</v>
       </c>
@@ -8354,9 +8435,9 @@
       <c r="H24" s="26"/>
       <c r="I24" s="24"/>
     </row>
-    <row r="25" spans="1:9" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="73"/>
-      <c r="B25" s="70"/>
+    <row r="25" spans="1:9" s="6" customFormat="1" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A25" s="94"/>
+      <c r="B25" s="91"/>
       <c r="C25" s="24">
         <v>7.4</v>
       </c>
@@ -8375,9 +8456,9 @@
       <c r="H25" s="26"/>
       <c r="I25" s="24"/>
     </row>
-    <row r="26" spans="1:9" s="6" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" s="6" customFormat="1" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A26" s="52"/>
-      <c r="B26" s="81"/>
+      <c r="B26" s="101"/>
       <c r="C26" s="24">
         <v>7.5</v>
       </c>
@@ -8396,11 +8477,11 @@
       <c r="H26" s="26"/>
       <c r="I26" s="24"/>
     </row>
-    <row r="27" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="78">
+    <row r="27" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="98">
         <v>8</v>
       </c>
-      <c r="B27" s="78" t="s">
+      <c r="B27" s="98" t="s">
         <v>44</v>
       </c>
       <c r="C27" s="28">
@@ -8423,9 +8504,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="79"/>
-      <c r="B28" s="79"/>
+    <row r="28" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="99"/>
+      <c r="B28" s="99"/>
       <c r="C28" s="28">
         <v>9.3000000000000007</v>
       </c>
@@ -8446,9 +8527,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="80"/>
-      <c r="B29" s="80"/>
+    <row r="29" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="100"/>
+      <c r="B29" s="100"/>
       <c r="C29" s="28">
         <v>9.4</v>
       </c>
@@ -8469,11 +8550,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="76">
+    <row r="30" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A30" s="96">
         <v>12</v>
       </c>
-      <c r="B30" s="76" t="s">
+      <c r="B30" s="96" t="s">
         <v>54</v>
       </c>
       <c r="C30" s="30">
@@ -8498,9 +8579,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="76"/>
-      <c r="B31" s="76"/>
+    <row r="31" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A31" s="96"/>
+      <c r="B31" s="96"/>
       <c r="C31" s="30">
         <v>12.2</v>
       </c>
@@ -8523,9 +8604,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="76"/>
-      <c r="B32" s="76"/>
+    <row r="32" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="96"/>
+      <c r="B32" s="96"/>
       <c r="C32" s="30">
         <v>12.3</v>
       </c>
@@ -8548,9 +8629,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:9" s="6" customFormat="1" ht="123.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="76"/>
-      <c r="B33" s="76"/>
+    <row r="33" spans="1:9" s="6" customFormat="1" ht="123.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="96"/>
+      <c r="B33" s="96"/>
       <c r="C33" s="30">
         <v>12.4</v>
       </c>
@@ -8573,9 +8654,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:9" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="76"/>
-      <c r="B34" s="76"/>
+    <row r="34" spans="1:9" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="96"/>
+      <c r="B34" s="96"/>
       <c r="C34" s="30">
         <v>12.5</v>
       </c>
@@ -8598,11 +8679,11 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="77">
+    <row r="35" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="97">
         <v>14</v>
       </c>
-      <c r="B35" s="77" t="s">
+      <c r="B35" s="97" t="s">
         <v>70</v>
       </c>
       <c r="C35" s="34">
@@ -8627,9 +8708,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="77"/>
-      <c r="B36" s="77"/>
+    <row r="36" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A36" s="97"/>
+      <c r="B36" s="97"/>
       <c r="C36" s="34">
         <v>14.2</v>
       </c>
@@ -8652,9 +8733,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A37" s="77"/>
-      <c r="B37" s="77"/>
+    <row r="37" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="97"/>
+      <c r="B37" s="97"/>
       <c r="C37" s="34">
         <v>14.3</v>
       </c>
@@ -8677,9 +8758,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="77"/>
-      <c r="B38" s="77"/>
+    <row r="38" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A38" s="97"/>
+      <c r="B38" s="97"/>
       <c r="C38" s="34">
         <v>14.4</v>
       </c>
@@ -8702,9 +8783,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="77"/>
-      <c r="B39" s="77"/>
+    <row r="39" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="97"/>
+      <c r="B39" s="97"/>
       <c r="C39" s="34">
         <v>14.5</v>
       </c>
@@ -8727,9 +8808,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="40" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A40" s="77"/>
-      <c r="B40" s="77"/>
+    <row r="40" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="97"/>
+      <c r="B40" s="97"/>
       <c r="C40" s="34">
         <v>14.6</v>
       </c>
@@ -8752,9 +8833,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="41" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A41" s="77"/>
-      <c r="B41" s="77"/>
+    <row r="41" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="97"/>
+      <c r="B41" s="97"/>
       <c r="C41" s="34">
         <v>14.7</v>
       </c>
@@ -8777,9 +8858,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="42" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A42" s="77"/>
-      <c r="B42" s="77"/>
+    <row r="42" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A42" s="97"/>
+      <c r="B42" s="97"/>
       <c r="C42" s="34">
         <v>14.8</v>
       </c>
@@ -8802,9 +8883,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="77"/>
-      <c r="B43" s="77"/>
+    <row r="43" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A43" s="97"/>
+      <c r="B43" s="97"/>
       <c r="C43" s="34">
         <v>14.9</v>
       </c>
@@ -8827,9 +8908,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="44" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="77"/>
-      <c r="B44" s="77"/>
+    <row r="44" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A44" s="97"/>
+      <c r="B44" s="97"/>
       <c r="C44" s="34">
         <v>14.1</v>
       </c>
@@ -8852,9 +8933,9 @@
         <v>72</v>
       </c>
     </row>
-    <row r="45" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A45" s="77"/>
-      <c r="B45" s="77"/>
+    <row r="45" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="97"/>
+      <c r="B45" s="97"/>
       <c r="C45" s="34">
         <v>14.11</v>
       </c>
@@ -8877,11 +8958,11 @@
         <v>72</v>
       </c>
     </row>
-    <row r="46" spans="1:9" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="74">
+    <row r="46" spans="1:9" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A46" s="95">
         <v>15</v>
       </c>
-      <c r="B46" s="74" t="s">
+      <c r="B46" s="95" t="s">
         <v>74</v>
       </c>
       <c r="C46" s="37">
@@ -8906,7 +8987,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="47" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A47" s="75"/>
       <c r="B47" s="75"/>
       <c r="C47" s="37">
@@ -8931,7 +9012,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A48" s="75"/>
       <c r="B48" s="75"/>
       <c r="C48" s="37">
@@ -8956,7 +9037,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="49" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A49" s="75"/>
       <c r="B49" s="75"/>
       <c r="C49" s="37">
@@ -8981,7 +9062,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A50" s="75"/>
       <c r="B50" s="75"/>
       <c r="C50" s="37">
@@ -9006,7 +9087,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A51" s="75"/>
       <c r="B51" s="75"/>
       <c r="C51" s="37">
@@ -9031,7 +9112,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="75"/>
       <c r="B52" s="75"/>
       <c r="C52" s="37">
@@ -9056,7 +9137,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="53" spans="1:9" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
       <c r="A53" s="75"/>
       <c r="B53" s="75"/>
       <c r="C53" s="37">
@@ -9081,11 +9162,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="54" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A54" s="97">
+    <row r="54" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A54" s="74">
         <v>16</v>
       </c>
-      <c r="B54" s="97" t="s">
+      <c r="B54" s="74" t="s">
         <v>89</v>
       </c>
       <c r="C54" s="39">
@@ -9110,9 +9191,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="55" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A55" s="97"/>
-      <c r="B55" s="97"/>
+    <row r="55" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A55" s="74"/>
+      <c r="B55" s="74"/>
       <c r="C55" s="39">
         <v>16.2</v>
       </c>
@@ -9135,9 +9216,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="56" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A56" s="97"/>
-      <c r="B56" s="97"/>
+    <row r="56" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A56" s="74"/>
+      <c r="B56" s="74"/>
       <c r="C56" s="39">
         <v>16.3</v>
       </c>
@@ -9160,9 +9241,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="57" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="97"/>
-      <c r="B57" s="97"/>
+    <row r="57" spans="1:9" s="6" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+      <c r="A57" s="74"/>
+      <c r="B57" s="74"/>
       <c r="C57" s="39">
         <v>16.399999999999999</v>
       </c>
@@ -9185,9 +9266,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="58" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A58" s="97"/>
-      <c r="B58" s="97"/>
+    <row r="58" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A58" s="74"/>
+      <c r="B58" s="74"/>
       <c r="C58" s="39">
         <v>16.5</v>
       </c>
@@ -9210,7 +9291,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="59" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A59" s="75"/>
       <c r="B59" s="75"/>
       <c r="C59" s="39">
@@ -9235,11 +9316,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="60" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="98">
+    <row r="60" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A60" s="76">
         <v>17</v>
       </c>
-      <c r="B60" s="101" t="s">
+      <c r="B60" s="79" t="s">
         <v>105</v>
       </c>
       <c r="C60" s="42">
@@ -9264,9 +9345,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="61" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A61" s="99"/>
-      <c r="B61" s="101"/>
+    <row r="61" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A61" s="77"/>
+      <c r="B61" s="79"/>
       <c r="C61" s="42">
         <v>17.2</v>
       </c>
@@ -9289,9 +9370,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="62" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="99"/>
-      <c r="B62" s="101"/>
+    <row r="62" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="77"/>
+      <c r="B62" s="79"/>
       <c r="C62" s="42">
         <v>17.3</v>
       </c>
@@ -9314,9 +9395,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A63" s="99"/>
-      <c r="B63" s="101"/>
+    <row r="63" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A63" s="77"/>
+      <c r="B63" s="79"/>
       <c r="C63" s="42">
         <v>17.399999999999999</v>
       </c>
@@ -9339,9 +9420,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="64" spans="1:9" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A64" s="100"/>
-      <c r="B64" s="101"/>
+    <row r="64" spans="1:9" s="6" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A64" s="78"/>
+      <c r="B64" s="79"/>
       <c r="C64" s="42">
         <v>17.5</v>
       </c>
@@ -9364,11 +9445,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="65" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A65" s="102">
+    <row r="65" spans="1:12" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A65" s="80">
         <v>18</v>
       </c>
-      <c r="B65" s="83" t="s">
+      <c r="B65" s="81" t="s">
         <v>279</v>
       </c>
       <c r="C65" s="18">
@@ -9393,9 +9474,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="66" spans="1:12" s="6" customFormat="1" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" s="6" customFormat="1" ht="250.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="75"/>
-      <c r="B66" s="84"/>
+      <c r="B66" s="82"/>
       <c r="C66" s="18">
         <v>18.2</v>
       </c>
@@ -9418,9 +9499,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="6" customFormat="1" ht="167.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" s="6" customFormat="1" ht="167.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="75"/>
-      <c r="B67" s="84"/>
+      <c r="B67" s="82"/>
       <c r="C67" s="18">
         <v>18.3</v>
       </c>
@@ -9443,9 +9524,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="68" spans="1:12" s="6" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" s="6" customFormat="1" ht="246.5" x14ac:dyDescent="0.35">
       <c r="A68" s="75"/>
-      <c r="B68" s="84"/>
+      <c r="B68" s="82"/>
       <c r="C68" s="18">
         <v>18.399999999999999</v>
       </c>
@@ -9468,9 +9549,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="6" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" s="6" customFormat="1" ht="216" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="48"/>
-      <c r="B69" s="85"/>
+      <c r="B69" s="83"/>
       <c r="C69" s="18">
         <v>18.5</v>
       </c>
@@ -9489,11 +9570,11 @@
       <c r="H69" s="18"/>
       <c r="I69" s="18"/>
     </row>
-    <row r="70" spans="1:12" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="91">
+    <row r="70" spans="1:12" s="6" customFormat="1" ht="87" x14ac:dyDescent="0.35">
+      <c r="A70" s="68">
         <v>19</v>
       </c>
-      <c r="B70" s="94" t="s">
+      <c r="B70" s="71" t="s">
         <v>120</v>
       </c>
       <c r="C70" s="44">
@@ -9514,9 +9595,9 @@
       <c r="H70" s="44"/>
       <c r="I70" s="47"/>
     </row>
-    <row r="71" spans="1:12" s="6" customFormat="1" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="92"/>
-      <c r="B71" s="95"/>
+    <row r="71" spans="1:12" s="6" customFormat="1" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A71" s="69"/>
+      <c r="B71" s="72"/>
       <c r="C71" s="15">
         <v>19.2</v>
       </c>
@@ -9535,9 +9616,9 @@
       <c r="H71" s="44"/>
       <c r="I71" s="47"/>
     </row>
-    <row r="72" spans="1:12" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="93"/>
-      <c r="B72" s="96"/>
+    <row r="72" spans="1:12" s="6" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A72" s="70"/>
+      <c r="B72" s="73"/>
       <c r="C72" s="53">
         <v>19.3</v>
       </c>
@@ -9558,11 +9639,11 @@
         <v>313</v>
       </c>
     </row>
-    <row r="73" spans="1:12" s="6" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A73" s="91">
+    <row r="73" spans="1:12" s="6" customFormat="1" ht="203" x14ac:dyDescent="0.35">
+      <c r="A73" s="68">
         <v>20</v>
       </c>
-      <c r="B73" s="94" t="s">
+      <c r="B73" s="71" t="s">
         <v>126</v>
       </c>
       <c r="C73" s="44">
@@ -9583,9 +9664,9 @@
       <c r="H73" s="44"/>
       <c r="I73" s="47"/>
     </row>
-    <row r="74" spans="1:12" s="6" customFormat="1" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A74" s="92"/>
-      <c r="B74" s="95"/>
+    <row r="74" spans="1:12" s="6" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A74" s="69"/>
+      <c r="B74" s="72"/>
       <c r="C74" s="15">
         <v>20.2</v>
       </c>
@@ -9607,9 +9688,9 @@
       <c r="K74" s="1"/>
       <c r="L74" s="1"/>
     </row>
-    <row r="75" spans="1:12" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A75" s="93"/>
-      <c r="B75" s="95"/>
+    <row r="75" spans="1:12" s="6" customFormat="1" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A75" s="70"/>
+      <c r="B75" s="72"/>
       <c r="C75" s="56">
         <v>20.3</v>
       </c>
@@ -9633,9 +9714,9 @@
       <c r="K75" s="1"/>
       <c r="L75" s="1"/>
     </row>
-    <row r="76" spans="1:12" s="6" customFormat="1" ht="331.2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" s="6" customFormat="1" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A76" s="49"/>
-      <c r="B76" s="96"/>
+      <c r="B76" s="73"/>
       <c r="C76" s="56">
         <v>20.399999999999999</v>
       </c>
@@ -9659,11 +9740,11 @@
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
     </row>
-    <row r="77" spans="1:12" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A77" s="91">
+    <row r="77" spans="1:12" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A77" s="68">
         <v>21</v>
       </c>
-      <c r="B77" s="94" t="s">
+      <c r="B77" s="71" t="s">
         <v>129</v>
       </c>
       <c r="C77" s="44">
@@ -9684,9 +9765,9 @@
       <c r="H77" s="44"/>
       <c r="I77" s="47"/>
     </row>
-    <row r="78" spans="1:12" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="92"/>
-      <c r="B78" s="95"/>
+    <row r="78" spans="1:12" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A78" s="69"/>
+      <c r="B78" s="72"/>
       <c r="C78" s="15">
         <v>21.2</v>
       </c>
@@ -9705,9 +9786,9 @@
       <c r="H78" s="44"/>
       <c r="I78" s="47"/>
     </row>
-    <row r="79" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A79" s="93"/>
-      <c r="B79" s="96"/>
+    <row r="79" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A79" s="70"/>
+      <c r="B79" s="73"/>
       <c r="C79" s="32">
         <v>21.3</v>
       </c>
@@ -9722,11 +9803,11 @@
       <c r="H79" s="32"/>
       <c r="I79" s="33"/>
     </row>
-    <row r="80" spans="1:12" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A80" s="91">
+    <row r="80" spans="1:12" ht="261" x14ac:dyDescent="0.35">
+      <c r="A80" s="68">
         <v>22</v>
       </c>
-      <c r="B80" s="94" t="s">
+      <c r="B80" s="71" t="s">
         <v>133</v>
       </c>
       <c r="C80" s="44">
@@ -9747,9 +9828,9 @@
       <c r="H80" s="44"/>
       <c r="I80" s="47"/>
     </row>
-    <row r="81" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
-      <c r="A81" s="92"/>
-      <c r="B81" s="95"/>
+    <row r="81" spans="1:9" ht="261" x14ac:dyDescent="0.35">
+      <c r="A81" s="69"/>
+      <c r="B81" s="72"/>
       <c r="C81" s="15">
         <v>22.2</v>
       </c>
@@ -9768,9 +9849,9 @@
       <c r="H81" s="44"/>
       <c r="I81" s="47"/>
     </row>
-    <row r="82" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A82" s="93"/>
-      <c r="B82" s="96"/>
+    <row r="82" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A82" s="70"/>
+      <c r="B82" s="73"/>
       <c r="C82" s="32">
         <v>22.3</v>
       </c>
@@ -9785,26 +9866,26 @@
       <c r="H82" s="32"/>
       <c r="I82" s="33"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="E83" s="11"/>
       <c r="H83" s="3"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="I84" s="2"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
       <c r="I85" s="2"/>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" s="7"/>
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
@@ -9815,7 +9896,7 @@
       <c r="H86" s="7"/>
       <c r="I86" s="7"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -9826,7 +9907,7 @@
       <c r="H87" s="10"/>
       <c r="I87" s="10"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D88" s="10"/>
       <c r="E88" s="10"/>
       <c r="F88" s="10"/>
@@ -9834,7 +9915,7 @@
       <c r="H88" s="10"/>
       <c r="I88" s="10"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="D89" s="10"/>
       <c r="E89" s="10"/>
@@ -9843,7 +9924,7 @@
       <c r="H89" s="10"/>
       <c r="I89" s="10"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D90" s="10"/>
       <c r="E90" s="10"/>
       <c r="F90" s="10"/>
@@ -9851,7 +9932,7 @@
       <c r="H90" s="10"/>
       <c r="I90" s="10"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D91" s="10"/>
       <c r="E91" s="10"/>
       <c r="F91" s="10"/>
@@ -9859,7 +9940,7 @@
       <c r="H91" s="10"/>
       <c r="I91" s="10"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D92" s="10"/>
       <c r="E92" s="10"/>
       <c r="F92" s="10"/>
@@ -9867,7 +9948,7 @@
       <c r="H92" s="10"/>
       <c r="I92" s="10"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D93" s="10"/>
       <c r="E93" s="10"/>
       <c r="F93" s="10"/>
@@ -9875,7 +9956,7 @@
       <c r="H93" s="10"/>
       <c r="I93" s="10"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D94" s="10"/>
       <c r="E94" s="10"/>
       <c r="F94" s="10"/>
@@ -9886,6 +9967,29 @@
   </sheetData>
   <autoFilter ref="I1:I32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="37">
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A46:A53"/>
+    <mergeCell ref="B46:B53"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="B30:B34"/>
+    <mergeCell ref="A35:A45"/>
+    <mergeCell ref="B35:B45"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B22:B26"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="A11:A15"/>
+    <mergeCell ref="B11:B15"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="B3:B10"/>
     <mergeCell ref="A77:A79"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A80:A82"/>
@@ -9900,29 +10004,6 @@
     <mergeCell ref="A73:A75"/>
     <mergeCell ref="B73:B76"/>
     <mergeCell ref="B65:B69"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="B11:B15"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A7"/>
-    <mergeCell ref="B3:B10"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A46:A53"/>
-    <mergeCell ref="B46:B53"/>
-    <mergeCell ref="A30:A34"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="A35:A45"/>
-    <mergeCell ref="B35:B45"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="B16:B21"/>
-    <mergeCell ref="B22:B26"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9934,15 +10015,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="18.21875" customWidth="1"/>
-    <col min="5" max="5" width="24.88671875" customWidth="1"/>
-    <col min="6" max="6" width="27.33203125" customWidth="1"/>
-    <col min="7" max="7" width="36.21875" customWidth="1"/>
+    <col min="4" max="4" width="18.1796875" customWidth="1"/>
+    <col min="5" max="5" width="24.90625" customWidth="1"/>
+    <col min="6" max="6" width="27.36328125" customWidth="1"/>
+    <col min="7" max="7" width="36.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="9"/>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -9954,7 +10035,7 @@
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="9"/>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
@@ -9966,7 +10047,7 @@
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
     </row>
-    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -9990,7 +10071,7 @@
       </c>
       <c r="J3" s="9"/>
     </row>
-    <row r="4" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="348" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
@@ -10014,7 +10095,7 @@
       </c>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="362.5" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
@@ -10038,7 +10119,7 @@
       </c>
       <c r="J5" s="9"/>
     </row>
-    <row r="6" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="348" x14ac:dyDescent="0.35">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
@@ -10062,7 +10143,7 @@
       </c>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:10" ht="403.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="406" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
@@ -10086,7 +10167,7 @@
       </c>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="333.5" x14ac:dyDescent="0.35">
       <c r="A8" s="9"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -10110,7 +10191,7 @@
       </c>
       <c r="J8" s="9"/>
     </row>
-    <row r="9" spans="1:10" ht="273.60000000000002" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A9" s="9"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -10134,7 +10215,7 @@
       </c>
       <c r="J9" s="9"/>
     </row>
-    <row r="10" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="348" x14ac:dyDescent="0.35">
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -10158,7 +10239,7 @@
       </c>
       <c r="J10" s="9"/>
     </row>
-    <row r="11" spans="1:10" ht="316.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="319" x14ac:dyDescent="0.35">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -10182,7 +10263,7 @@
       </c>
       <c r="J11" s="9"/>
     </row>
-    <row r="12" spans="1:10" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -10206,7 +10287,7 @@
       </c>
       <c r="J12" s="9"/>
     </row>
-    <row r="13" spans="1:10" ht="388.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -10230,7 +10311,7 @@
       </c>
       <c r="J13" s="9"/>
     </row>
-    <row r="14" spans="1:10" ht="288" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="290" x14ac:dyDescent="0.35">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -10254,7 +10335,7 @@
       </c>
       <c r="J14" s="9"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -10266,7 +10347,7 @@
       <c r="I15" s="9"/>
       <c r="J15" s="9"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -10278,7 +10359,7 @@
       <c r="I16" s="9"/>
       <c r="J16" s="9"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -10290,7 +10371,7 @@
       <c r="I17" s="9"/>
       <c r="J17" s="9"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="9"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -10302,7 +10383,7 @@
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
@@ -10314,7 +10395,7 @@
       <c r="I19" s="9"/>
       <c r="J19" s="9"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -10326,7 +10407,7 @@
       <c r="I20" s="9"/>
       <c r="J20" s="9"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
@@ -10338,7 +10419,7 @@
       <c r="I21" s="9"/>
       <c r="J21" s="9"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
@@ -10350,7 +10431,7 @@
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
@@ -10362,7 +10443,7 @@
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="9"/>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
@@ -10374,7 +10455,7 @@
       <c r="I24" s="9"/>
       <c r="J24" s="9"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="9"/>
       <c r="B25" s="9"/>
       <c r="C25" s="9"/>
@@ -10386,7 +10467,7 @@
       <c r="I25" s="9"/>
       <c r="J25" s="9"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="9"/>
       <c r="B26" s="9"/>
       <c r="C26" s="9"/>
@@ -10398,7 +10479,7 @@
       <c r="I26" s="9"/>
       <c r="J26" s="9"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>
@@ -10410,7 +10491,7 @@
       <c r="I27" s="9"/>
       <c r="J27" s="9"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="9"/>
       <c r="B28" s="9"/>
       <c r="C28" s="9"/>
@@ -10422,7 +10503,7 @@
       <c r="I28" s="9"/>
       <c r="J28" s="9"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="9"/>
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
@@ -10434,7 +10515,7 @@
       <c r="I29" s="9"/>
       <c r="J29" s="9"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="9"/>
       <c r="B30" s="9"/>
       <c r="C30" s="9"/>
@@ -10446,7 +10527,7 @@
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="9"/>
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
@@ -10458,7 +10539,7 @@
       <c r="I31" s="9"/>
       <c r="J31" s="9"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="9"/>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -10470,63 +10551,63 @@
       <c r="I32" s="9"/>
       <c r="J32" s="9"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="9"/>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
       <c r="E33" s="9"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="9"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
       <c r="E34" s="9"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="9"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="9"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="9"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="9"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
       <c r="E37" s="9"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="9"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="9"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
       <c r="E39" s="9"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="9"/>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="9"/>
       <c r="B41" s="9"/>
       <c r="C41" s="9"/>
@@ -10542,33 +10623,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0802363A-09BC-4F89-B136-783D2DDEAFD1}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.77734375" customWidth="1"/>
-    <col min="2" max="2" width="43.5546875" customWidth="1"/>
-    <col min="3" max="3" width="55.21875" customWidth="1"/>
-    <col min="4" max="4" width="70.21875" customWidth="1"/>
-    <col min="5" max="5" width="89.77734375" customWidth="1"/>
+    <col min="1" max="1" width="21.81640625" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" customWidth="1"/>
+    <col min="3" max="3" width="55.1796875" customWidth="1"/>
+    <col min="4" max="4" width="70.1796875" customWidth="1"/>
+    <col min="5" max="5" width="89.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="68" t="s">
+    <row r="1" spans="1:5" ht="37.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="67" t="s">
         <v>332</v>
       </c>
-      <c r="B1" s="68" t="s">
+      <c r="B1" s="67" t="s">
         <v>333</v>
       </c>
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="67" t="s">
         <v>334</v>
       </c>
-      <c r="D1" s="68" t="s">
+      <c r="D1" s="67" t="s">
         <v>335</v>
       </c>
-      <c r="E1" s="68" t="s">
+      <c r="E1" s="67" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="144" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="145" x14ac:dyDescent="0.35">
       <c r="A2" s="58">
         <v>5.0999999999999996</v>
       </c>
@@ -10585,7 +10666,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A3" s="58">
         <v>5.2</v>
       </c>
@@ -10602,7 +10683,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A4" s="58">
         <v>5.3</v>
       </c>
@@ -10619,7 +10700,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A5" s="58">
         <v>5.4</v>
       </c>
@@ -10636,7 +10717,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A6" s="61">
         <v>5.5</v>
       </c>
@@ -10649,11 +10730,11 @@
       <c r="D6" s="62" t="s">
         <v>348</v>
       </c>
-      <c r="E6" s="63" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="E6" s="102" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A7" s="58">
         <v>5.6</v>
       </c>
@@ -10667,27 +10748,27 @@
         <v>351</v>
       </c>
       <c r="E7" s="60" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="64">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A8" s="63">
         <v>5.7</v>
       </c>
-      <c r="B8" s="65" t="s">
+      <c r="B8" s="64" t="s">
         <v>352</v>
       </c>
-      <c r="C8" s="65" t="s">
+      <c r="C8" s="64" t="s">
         <v>353</v>
       </c>
-      <c r="D8" s="66" t="s">
-        <v>373</v>
-      </c>
-      <c r="E8" s="64" t="s">
+      <c r="D8" s="65" t="s">
+        <v>371</v>
+      </c>
+      <c r="E8" s="63" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A9" s="58">
         <v>5.8</v>
       </c>
@@ -10704,7 +10785,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A10" s="58">
         <v>5.9</v>
       </c>
@@ -10721,8 +10802,8 @@
         <v>366</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="144" x14ac:dyDescent="0.3">
-      <c r="A11" s="67">
+    <row r="11" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A11" s="66">
         <v>5.0999999999999996</v>
       </c>
       <c r="B11" s="59" t="s">

</xml_diff>